<commit_message>
Vérification manuelle : expertAtlas, Coaching Financement Pacte Industrie, AKTO bilan compétences
- expertAtlas (Atlas) : taux confirmé (jusqu'à 100%, sous conditions) + note
  plafond de minimis (300k€/3 ans) + lien corrigé vers la fiche produit.
- Coaching Financement décarbonation (Pacte Industrie) : taux confirmé à 80%
  et durée (2 à 5 jours) trouvés sur la page officielle.
- akto_proprete_bilan_competences : le taux 9,15€/h ne correspond plus à
  aucune section "Bilan de compétences" dans les Règles de prise en charge
  AKTO 2026 (probablement une confusion avec la ligne "période de
  reconversion" du même document) — repassé en N/A à reconfirmer plutôt que
  de garder un chiffre non sourcé.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCES.xlsx
+++ b/SOURCES.xlsx
@@ -942,22 +942,22 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>N/A — à vérifier sur opco-atlas.fr</t>
+          <t>Jusqu'à 100 % du coût de la prestation (Atlas + État), sous conditions</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>N/A — à vérifier sur opco-atlas.fr</t>
+          <t>N/A — soumis au plafond de minimis (300 000 € d'aides publiques sur 3 exercices fiscaux)</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>https://www.opco-atlas.fr/criteres-financement/</t>
+          <t>https://www.opco-atlas.fr/entreprise/accompagnement-ressources-humaines.html</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -2312,12 +2312,12 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>9,15 €/h</t>
+          <t>N/A — non retrouvé dans les Règles de prise en charge 2026, à reconfirmer auprès d'AKTO</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Selon durée du bilan</t>
+          <t>N/A — à reconfirmer auprès d'AKTO</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Prise en charge du bilan de compétences pour les salariés de la branche Propreté. Forfait horaire fixe.</t>
+          <t>Prise en charge du bilan de compétences pour les salariés de la branche Propreté. ATTENTION : aucune section \</t>
         </is>
       </c>
     </row>
@@ -7004,7 +7004,7 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>N/A — barème non confirmé pour ce dispositif précis, à vérifier sur pacte-industrie.ademe.fr</t>
+          <t>Financé jusqu'à 80 % du prix de l'accompagnement</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ajoute 4 aides régionales phares hors Île-de-France
Auvergne-Rhône-Alpes, Hauts-de-France, Nouvelle-Aquitaine : une aide
transition écologique/décarbonation par région (2 pour la Nouvelle-
Aquitaine), pour amorcer une couverture nationale plus équilibrée.
Périmètre volontairement limité (1-2 aides/région) pour contenir le coût
de recherche ; FRATRI (Hauts-de-France) et FNVI écartés car non
directement actionnables par une entreprise (enveloppes globales/
fonds de fonds, pas des aides à guichet individuel).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCES.xlsx
+++ b/SOURCES.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procédure MAJ" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aides'!$A$1:$M$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aides'!$A$1:$M$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7264,8 +7264,260 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>ara_financement_energie</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>TEE</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Financer des projets innovants et/ou expérimentaux autour de l'énergie — Région Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Région Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>30 % maximum des dépenses d'investissement HT</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>N/A — voir dossier de candidature</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.auvergnerhonealpes.fr/aides/financer-des-projets-innovants-etou-experimentaux-autour-de-lenergie</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>Soutien aux projets de solutions décarbonées, énergies renouvelables, stockage/conversion énergétique, captage-valorisation du CO2 et réseaux intelligents. Ouvert à tous types de maîtres d'ouvrage hors particuliers et État.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>hdf_btr3</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>TEE</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Booster Transformation Rev3 (BTR3) — Région Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Région Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>50 % du coût HT de la mission</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>10 000 € par facture payée (maximum 2 missions/an sur des modules différents)</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>https://guide-aides.hautsdefrance.fr/dispositif1045</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>Aide au financement de missions d'accompagnement (diagnostic/conseil) sur la transition économique, énergétique et environnementale des PME : efficacité énergétique, économie circulaire, bilan carbone, adaptation climatique (7 modules).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>na_usine_du_futur</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>TEE</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Usine du Futur — Région Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Région Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>100 % pris en charge par la Région</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Prestation gratuite pour l'entreprise</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>https://les-aides.nouvelle-aquitaine.fr/transition-energetique-et-ecologique/usine-du-futur-agissons-aujourd-hui-pour-une-industrie-durable-et-competitive</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>Diagnostic terrain et accompagnement méthodologique des PME/ETI industrielles sur 5 leviers (stratégie, industrie, collectif, donnée, technologie), avec une dimension décarbonation/environnementale croissante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>na_competitivite_energetique</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>TEE</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Compétitivité énergétique des entreprises — Région Nouvelle-Aquitaine</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Région Nouvelle-Aquitaine (cofinancement possible FEDER)</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>N/A — taux non publié sur la fiche, à vérifier (règlement PDF non consulté)</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>N/A — voir les-aides.nouvelle-aquitaine.fr</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>https://les-aides.nouvelle-aquitaine.fr/economie-et-emploi/competitivite-energetique-des-entreprises</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>Soutien aux entreprises industrielles pour des études (audits, faisabilité) et des investissements visant l'efficacité énergétique et les énergies renouvelables dans les procédés, avec un objectif minimum de 10 % de réduction de la consommation d'énergie du site. Cofinancement possible FEDER.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M110"/>
+  <autoFilter ref="A1:M114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>